<commit_message>
testes versao pudim em andamento - com e sem pca + monte carlo
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/dados_teste/fornax/DADOS_FORNAX.xlsx
+++ b/V. 2 (Pudim)/dados_teste/fornax/DADOS_FORNAX.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Documents\dev\Finscore\FinScore\jupyter\fornax\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Documents\dev\Finscore\FinScore\V. 2 (Pudim)\dados_teste\fornax\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B263202-A1B9-4218-9B76-8D1B39C9BAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3AFDC5-763D-4376-9DB8-D1E2E3C12A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="lancamentos" sheetId="1" r:id="rId1"/>
     <sheet name="NOTA_TECNICA" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -147,12 +147,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -167,8 +179,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,25 +511,25 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
@@ -533,13 +547,13 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Q1" t="s">
@@ -550,25 +564,25 @@
       <c r="A2">
         <v>2025</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>10061764.119999999</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>10178773.52</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="2">
         <v>725788.67</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
         <v>618.75</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="2">
         <v>8665337.2400000002</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="2">
         <v>5258385.4000000004</v>
       </c>
       <c r="I2">
@@ -586,13 +600,13 @@
       <c r="M2">
         <v>0</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="1">
         <v>5645884.5800000001</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="2">
         <v>998713.91</v>
       </c>
-      <c r="P2">
+      <c r="P2" s="1">
         <v>11736317.970000001</v>
       </c>
       <c r="Q2">
@@ -603,25 +617,25 @@
       <c r="A3">
         <v>2024</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>8716303.9700000007</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>8833313.3699999992</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>896040.65</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
         <v>6543935</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="2">
         <v>3220520.14</v>
       </c>
       <c r="I3">
@@ -639,13 +653,13 @@
       <c r="M3">
         <v>457.53</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="1">
         <v>4991722.7300000004</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="2">
         <v>13600.33</v>
       </c>
-      <c r="P3">
+      <c r="P3" s="1">
         <v>14211992.210000001</v>
       </c>
       <c r="Q3">
@@ -656,25 +670,25 @@
       <c r="A4">
         <v>2023</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>4844724.01</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>4845181.54</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>2679999.73</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
         <v>1088677.93</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="2">
         <v>3587160.8</v>
       </c>
       <c r="I4">
@@ -692,13 +706,13 @@
       <c r="M4">
         <v>0</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="1">
         <v>4030997.57</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="2">
         <v>11543.78</v>
       </c>
-      <c r="P4">
+      <c r="P4" s="1">
         <v>9768495</v>
       </c>
       <c r="Q4">

</xml_diff>